<commit_message>
Actualización funcionamiento y comprobación de cambio de posición de muestras por excel.
</commit_message>
<xml_diff>
--- a/bateria_tests/cambio_pos_muestras/plantilla_cambio_posicion.xlsx
+++ b/bateria_tests/cambio_pos_muestras/plantilla_cambio_posicion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\OneDrive\Documentos\Practicas_UOC\datos_muestras\bateria_tests\cambio_pos_muestras\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mthem\Desktop\programas_python\datos_prueba\datos_prueba\globalstaticfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5651647-5671-4AF1-BD54-B108DE34460B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4B6F27-2970-4804-A352-1D78FAD7E973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Nombre Laboratorio</t>
   </si>
@@ -49,15 +52,6 @@
   </si>
   <si>
     <t>Subposición</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>EPSILON</t>
-  </si>
-  <si>
-    <t>loc_15</t>
   </si>
 </sst>
 </file>
@@ -384,20 +378,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.81640625" customWidth="1"/>
-    <col min="8" max="8" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -421,32 +415,6 @@
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>